<commit_message>
Update bulk upload point
</commit_message>
<xml_diff>
--- a/data/bulk-upload-points/upload-points-invalid-data.xlsx
+++ b/data/bulk-upload-points/upload-points-invalid-data.xlsx
@@ -1,29 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cabe-1078\Desktop\Noted_CAB_2026\Data_Test_WUPoint\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CF4DC16-2132-4012-B474-5DCB75C76026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C024229E-C56A-45BA-B966-A2E7BFEFB345}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="data" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
-  <si>
-    <t>no</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
   <si>
     <t>cifId</t>
   </si>
@@ -64,19 +75,25 @@
     <t>description</t>
   </si>
   <si>
-    <t>RECEIVE_MONEY</t>
-  </si>
-  <si>
-    <t>BRANCH</t>
-  </si>
-  <si>
-    <t>TRANSFER_MONEY</t>
-  </si>
-  <si>
-    <t>MOBILE_BANKING</t>
-  </si>
-  <si>
     <t>remark:</t>
+  </si>
+  <si>
+    <t>Transfer Money</t>
+  </si>
+  <si>
+    <t>Receive Money</t>
+  </si>
+  <si>
+    <t>Mobile Banking</t>
+  </si>
+  <si>
+    <t>Branch</t>
+  </si>
+  <si>
+    <t>PASSPORT</t>
+  </si>
+  <si>
+    <t>NID</t>
   </si>
 </sst>
 </file>
@@ -105,7 +122,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -113,30 +130,17 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -439,85 +443,124 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.21875" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="8" max="8" width="10.77734375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3" s="2"/>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A5" s="2"/>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A7" s="2"/>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>2</v>
+      </c>
+      <c r="D9" t="s">
+        <v>3</v>
+      </c>
+      <c r="E9" t="s">
+        <v>4</v>
+      </c>
+      <c r="F9" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="G9" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H7" s="1" t="s">
+      <c r="H9" t="s">
         <v>7</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="I9" t="s">
         <v>8</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="J9" t="s">
         <v>9</v>
       </c>
-      <c r="K7" s="1" t="s">
+      <c r="K9" t="s">
         <v>10</v>
       </c>
-      <c r="L7" s="1" t="s">
+      <c r="L9" t="s">
         <v>11</v>
       </c>
-      <c r="M7" s="1" t="s">
+      <c r="M9" t="s">
         <v>12</v>
       </c>
-      <c r="N7" s="1" t="s">
-        <v>13</v>
-      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A10" s="3"/>
+      <c r="D10" s="3"/>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A7"/>
+  </mergeCells>
+  <dataValidations count="3">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Invalid Value" error="Please select from dropdown only." sqref="G10:G100" xr:uid="{3A73E993-6E85-4028-9A03-04AECBCF2D11}">
+      <formula1>"PASSPORT,NID"</formula1>
+    </dataValidation>
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Invalid Value" error="Please select from dropdown only." sqref="F10:F100" xr:uid="{B88F7665-AECC-41D8-97E5-0651A7827F53}">
+      <formula1>"Mobile Banking,Branch"</formula1>
+    </dataValidation>
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Invalid Value" error="Please select from dropdown only." sqref="E10:E100" xr:uid="{35705B6C-AEC3-4CE8-924A-6304695D0C2A}">
+      <formula1>"Transfer Money,Receive Money"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>